<commit_message>
errr new resources parts list
</commit_message>
<xml_diff>
--- a/Electrical/PCB v1/L1/Parts List L1 V1.xlsx
+++ b/Electrical/PCB v1/L1/Parts List L1 V1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ad0bf7e61e147d2/Documents/GitHub/robocup2025/Electronics/PCB v1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ad0bf7e61e147d2/Documents/GitHub/robocup2025/Electrical/PCB v1/L1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{643554D1-2880-42A2-825E-C6D10EA67947}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EC9E935-3E8C-4D03-AA79-1CD4E62C8F3D}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22276" windowHeight="13276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13133" yWindow="0" windowWidth="9030" windowHeight="13163" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t xml:space="preserve">Parts list </t>
   </si>
@@ -74,9 +74,6 @@
     <t>https://www.lcsc.com/datasheet/lcsc_datasheet_1806131537_Everlight-Elec-ALS-PT19-315C-L177-TR8_C146233.pdf</t>
   </si>
   <si>
-    <t>refer to ducc boat</t>
-  </si>
-  <si>
     <t>refer to ducc</t>
   </si>
   <si>
@@ -92,9 +89,6 @@
     <t>no clue</t>
   </si>
   <si>
-    <t>soh</t>
-  </si>
-  <si>
     <t>https://www.snapeda.com/parts/ESP32-S3-WROOM-1-N16R8/Espressif%20Systems/datasheet/</t>
   </si>
   <si>
@@ -102,6 +96,15 @@
   </si>
   <si>
     <t>SM0603UYC</t>
+  </si>
+  <si>
+    <t>0.8 x 0.6 x 1.7</t>
+  </si>
+  <si>
+    <t>50 mm x 25 mm x (8-10) mm</t>
+  </si>
+  <si>
+    <t>1.6mm x 08mm x 0.6 mm</t>
   </si>
 </sst>
 </file>
@@ -176,10 +179,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -451,7 +450,7 @@
     <col min="1" max="1" width="11.265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.19921875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.06640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.9296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="102.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -489,22 +488,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F4" s="1">
         <v>20</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
@@ -512,16 +511,16 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1">
         <v>0.05</v>
@@ -532,13 +531,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
       </c>
       <c r="F6">
         <v>0.05</v>

</xml_diff>